<commit_message>
Busca la tabla de seguimiento en la hoja Flujos y en cualquier fila; ficticio gemelo del real
</commit_message>
<xml_diff>
--- a/data/ejemplo/casos_ficticios.xlsx
+++ b/data/ejemplo/casos_ficticios.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Seguimiento" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flujos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,6 +430,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Resumen del seguimiento — DATOS FICTICIOS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AE67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>